<commit_message>
docs(qa): separate Faculty Governance and Academic Affairs into dedicated sheets with 187 comprehensive test cases
</commit_message>
<xml_diff>
--- a/PROGROUP_AI_TESTCASES_DAY_DU_CHI_TIET.xlsx
+++ b/PROGROUP_AI_TESTCASES_DAY_DU_CHI_TIET.xlsx
@@ -10,17 +10,18 @@
     <sheet name="2. Xác thực &amp; Hệ thống" sheetId="1" r:id="rId1"/>
     <sheet name="3. Phân hệ Sinh viên" sheetId="2" r:id="rId2"/>
     <sheet name="4. Phân hệ Giảng viên" sheetId="3" r:id="rId3"/>
-    <sheet name="5. Giáo vụ &amp; Đào tạo" sheetId="4" r:id="rId4"/>
-    <sheet name="6. Quản trị hệ thống" sheetId="5" r:id="rId5"/>
-    <sheet name="7. Phi chức năng &amp; Bảo mật" sheetId="6" r:id="rId6"/>
-    <sheet name="1. Tổng quan &amp; Dashboard" sheetId="7" r:id="rId7"/>
+    <sheet name="5. Giáo vụ khoa" sheetId="4" r:id="rId4"/>
+    <sheet name="6. Phòng đào tạo" sheetId="5" r:id="rId5"/>
+    <sheet name="7. Quản trị hệ thống" sheetId="6" r:id="rId6"/>
+    <sheet name="8. Phi chức năng &amp; Bảo mật" sheetId="7" r:id="rId7"/>
+    <sheet name="1. Tổng quan &amp; Dashboard" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1840" uniqueCount="1276">
   <si>
     <t>📋 KỊCH BẢN KIỂM THỬ PHÂN HỆ XÁC THỰC &amp; CÀI ĐẶT HỆ THỐNG</t>
   </si>
@@ -2133,75 +2134,127 @@
     <t>Hiển thị đầy đủ danh sách nhóm kèm điểm từng giai đoạn và điểm trung bình tiến độ.</t>
   </si>
   <si>
-    <t>📋 KỊCH BẢN KIỂM THỬ PHÂN HỆ GIÁO VỤ KHOA &amp; PHÒNG ĐÀO TẠO</t>
-  </si>
-  <si>
-    <t>TC_GOV_001</t>
-  </si>
-  <si>
-    <t>Tổng quan Khoa</t>
-  </si>
-  <si>
-    <t>Xem số liệu thống kê đào tạo tổng thể toàn khoa</t>
-  </si>
-  <si>
-    <t>Đăng nhập gvk.demo.</t>
+    <t>📋 KỊCH BẢN KIỂM THỬ PHÂN HỆ GIÁO VỤ KHOA (FACULTY GOVERNANCE)</t>
+  </si>
+  <si>
+    <t>TC_GVK_001</t>
+  </si>
+  <si>
+    <t>Dashboard Khoa</t>
+  </si>
+  <si>
+    <t>Hiển thị số liệu tổng quan đào tạo của khoa CNTT</t>
+  </si>
+  <si>
+    <t>Đăng nhập tài khoản gvk.demo.</t>
   </si>
   <si>
     <t>1. Vào Dashboard Giáo vụ khoa.
-2. Quan sát các Stat Card 4 màu.</t>
+2. Quan sát các Stat Card.</t>
   </si>
   <si>
     <t>GET /api/admin/overview</t>
   </si>
   <si>
-    <t>Hiển thị chính xác: Tổng số LHP khoa, Tổng số SV khoa, Tổng số GV khoa, Tổng số nhóm đồ án.</t>
-  </si>
-  <si>
-    <t>TC_GOV_002</t>
+    <t>Hiển thị đúng tổng số: LHP thuộc khoa, Số sinh viên khoa, Số giảng viên khoa, Số nhóm đồ án đang hoạt động.</t>
+  </si>
+  <si>
+    <t>TC_GVK_002</t>
+  </si>
+  <si>
+    <t>Làm mới dữ liệu Dashboard khoa bằng thao tác kéo (Pull-to-refresh)</t>
+  </si>
+  <si>
+    <t>Tại Dashboard Giáo vụ.</t>
+  </si>
+  <si>
+    <t>1. Kéo màn hình từ trên xuống dưới.
+2. Thả tay để reload.</t>
+  </si>
+  <si>
+    <t>Pull-to-refresh</t>
+  </si>
+  <si>
+    <t>Icon loading xoay tròn, tải lại số liệu mới nhất từ CSDL thành công.</t>
+  </si>
+  <si>
+    <t>TC_GVK_003</t>
   </si>
   <si>
     <t>Quản lý LHP</t>
   </si>
   <si>
-    <t>Xem danh mục toàn bộ các Lớp học phần của khoa</t>
-  </si>
-  <si>
-    <t>Đang ở quyền Giáo vụ khoa.</t>
+    <t>Xem danh mục tất cả Lớp học phần do Khoa quản lý</t>
+  </si>
+  <si>
+    <t>Khoa có ít nhất 3 LHP được mở.</t>
   </si>
   <si>
     <t>1. Vào tab 'Quản lý LHP'.
-2. Xem danh sách các LHP.</t>
+2. Quan sát danh sách card LHP.</t>
   </si>
   <si>
     <t>GET /api/lop-hoc-phan</t>
   </si>
   <si>
-    <t>Hiển thị danh sách card LHP: Mã lớp, Tên môn học, Học kỳ, Giảng viên phụ trách, Tình trạng phân công.</t>
-  </si>
-  <si>
-    <t>TC_GOV_003</t>
+    <t>Hiển thị đầy đủ: Mã lớp, Tên môn học, Học kỳ, Tên giảng viên phụ trách, Tình trạng phân công, Sĩ số sinh viên.</t>
+  </si>
+  <si>
+    <t>TC_GVK_004</t>
   </si>
   <si>
     <t>Tìm kiếm LHP</t>
   </si>
   <si>
-    <t>Tìm kiếm LHP theo Mã hoặc Tên môn trong khoa</t>
-  </si>
-  <si>
-    <t>Tại màn hình LHP của Giáo vụ.</t>
-  </si>
-  <si>
-    <t>1. Nhập 'Lập trình' vào ô tìm kiếm.</t>
-  </si>
-  <si>
-    <t>Search: 'Lập trình'</t>
-  </si>
-  <si>
-    <t>Lọc chính xác các môn có chứa từ khóa 'Lập trình'.</t>
-  </si>
-  <si>
-    <t>TC_GOV_004</t>
+    <t>Tìm kiếm LHP theo Mã môn hoặc Tên môn trong khoa</t>
+  </si>
+  <si>
+    <t>Tại danh sách LHP của Giáo vụ.</t>
+  </si>
+  <si>
+    <t>1. Nhập từ khóa 'Di động' vào ô tìm kiếm.
+2. Nhập mã môn 'IT301'.</t>
+  </si>
+  <si>
+    <t>Search: 'Di động' / 'IT301'</t>
+  </si>
+  <si>
+    <t>Danh sách lập tức lọc chính xác các LHP khớp từ khóa tìm kiếm.</t>
+  </si>
+  <si>
+    <t>TC_GVK_005</t>
+  </si>
+  <si>
+    <t>Lọc LHP</t>
+  </si>
+  <si>
+    <t>Lọc danh sách LHP theo Học kỳ niên khóa</t>
+  </si>
+  <si>
+    <t>1. Chọn lọc theo 'Học kỳ 1 2026-2027'.
+2. Chọn lọc theo 'Học kỳ 2 2026-2027'.</t>
+  </si>
+  <si>
+    <t>Filter by Semester</t>
+  </si>
+  <si>
+    <t>Chỉ hiển thị các LHP được mở trong học kỳ đã chọn.</t>
+  </si>
+  <si>
+    <t>TC_GVK_006</t>
+  </si>
+  <si>
+    <t>Xem thông tin chi tiết một LHP khoa (Danh sách SV và Nhóm)</t>
+  </si>
+  <si>
+    <t>1. Bấm vào một LHP cụ thể.
+2. Xem chi tiết danh sách sinh viên ghi danh và các nhóm đồ án.</t>
+  </si>
+  <si>
+    <t>Hiển thị đầy đủ danh sách sinh viên trong lớp, danh sách các nhóm đã thành lập và đề tài tương ứng.</t>
+  </si>
+  <si>
+    <t>TC_GVK_007</t>
   </si>
   <si>
     <t>Phân công GV</t>
@@ -2210,7 +2263,7 @@
     <t>Phân công Giảng viên phụ trách Lớp học phần thành công</t>
   </si>
   <si>
-    <t>Có LHP chưa có giảng viên phụ trách.</t>
+    <t>Có LHP chưa được phân công giảng viên.</t>
   </si>
   <si>
     <t>1. Vào mục 'Phân công giảng viên'.
@@ -2222,33 +2275,140 @@
     <t>POST /api/governance/assignments</t>
   </si>
   <si>
-    <t>Phân công thành công, giảng viên được gán vào LHP và có quyền quản lý đợt đồ án của lớp.</t>
-  </si>
-  <si>
-    <t>TC_GOV_005</t>
+    <t>Phân công thành công, hiển thị tên Giảng viên trên card LHP và gửi thông báo tới tài khoản GV.</t>
+  </si>
+  <si>
+    <t>TC_GVK_008</t>
+  </si>
+  <si>
+    <t>Chặn phân công trùng lặp cùng 1 giảng viên 2 lần vào 1 LHP</t>
+  </si>
+  <si>
+    <t>GV A đã được phân công vào LHP X.</t>
+  </si>
+  <si>
+    <t>1. Thử chọn lại GV A để phân công vào LHP X lần nữa.</t>
+  </si>
+  <si>
+    <t>Duplicate assignment</t>
+  </si>
+  <si>
+    <t>Hệ thống báo cảnh báo: 'Giảng viên này đã được phân công cho lớp học phần từ trước'.</t>
+  </si>
+  <si>
+    <t>TC_GVK_009</t>
+  </si>
+  <si>
+    <t>Đổi phân công</t>
+  </si>
+  <si>
+    <t>Thay đổi Giảng viên phụ trách LHP sang Giảng viên khác</t>
+  </si>
+  <si>
+    <t>LHP đang có GV A phụ trách.</t>
+  </si>
+  <si>
+    <t>1. Chọn LHP cần đổi GV.
+2. Bấm 'Đổi giảng viên'.
+3. Chọn GV B và bấm Xác nhận.</t>
+  </si>
+  <si>
+    <t>PUT /api/governance/assignments</t>
+  </si>
+  <si>
+    <t>Cập nhật thành công GV B phụ trách lớp. GV B đăng nhập vào sẽ thấy lớp này.</t>
+  </si>
+  <si>
+    <t>TC_GVK_010</t>
   </si>
   <si>
     <t>Hủy phân công</t>
   </si>
   <si>
-    <t>Hủy phân công hoặc đổi Giảng viên phụ trách LHP</t>
-  </si>
-  <si>
-    <t>LHP đã có GV được phân công.</t>
-  </si>
-  <si>
-    <t>1. Chọn LHP cần đổi GV.
-2. Chọn 'Đổi giảng viên phụ trách'.
-3. Chọn GV mới và xác nhận.</t>
-  </si>
-  <si>
-    <t>PUT /api/governance/assignments</t>
-  </si>
-  <si>
-    <t>Cập nhật thành công giảng viên mới phụ trách lớp.</t>
-  </si>
-  <si>
-    <t>TC_GOV_006</t>
+    <t>Hủy phân công giảng viên khỏi LHP khi chưa có nhóm đăng ký</t>
+  </si>
+  <si>
+    <t>LHP chưa bắt đầu làm đồ án.</t>
+  </si>
+  <si>
+    <t>1. Chọn 'Hủy phân công giảng viên'.
+2. Xác nhận hủy.</t>
+  </si>
+  <si>
+    <t>DELETE /api/governance/assignments</t>
+  </si>
+  <si>
+    <t>Hủy thành công, LHP quay về trạng thái 'Chưa phân công giảng viên'.</t>
+  </si>
+  <si>
+    <t>TC_GVK_011</t>
+  </si>
+  <si>
+    <t>Đồng bộ GV</t>
+  </si>
+  <si>
+    <t>Kiểm tra Giảng viên được phân công thấy lớp ngay trên tài khoản của mình</t>
+  </si>
+  <si>
+    <t>Vừa phân công GV A vào LHP mới.</t>
+  </si>
+  <si>
+    <t>1. Đăng xuất tài khoản Giáo vụ.
+2. Đăng nhập tài khoản GV A.
+3. Kiểm tra tab 'Lớp học phần'.</t>
+  </si>
+  <si>
+    <t>User: gv001</t>
+  </si>
+  <si>
+    <t>LHP mới lập tức xuất hiện trong danh sách phụ trách của Giảng viên A.</t>
+  </si>
+  <si>
+    <t>TC_GVK_012</t>
+  </si>
+  <si>
+    <t>Giám sát đăng ký</t>
+  </si>
+  <si>
+    <t>Xem màn hình Giám sát tổng quan đăng ký đồ án toàn khoa</t>
+  </si>
+  <si>
+    <t>Tại menu Giáo vụ.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Giám sát đăng ký đồ án'.
+2. Quan sát bảng số liệu.</t>
+  </si>
+  <si>
+    <t>GET /api/dang-ky-de-tai</t>
+  </si>
+  <si>
+    <t>Hiển thị tổng số nhóm đã đăng ký, số nhóm đã được duyệt, số nhóm chưa có đề tài theo từng môn.</t>
+  </si>
+  <si>
+    <t>TC_GVK_013</t>
+  </si>
+  <si>
+    <t>Thống kê đề tài</t>
+  </si>
+  <si>
+    <t>Xem báo cáo danh mục đề tài toàn khoa theo từng bộ môn</t>
+  </si>
+  <si>
+    <t>Có nhiều đề tài đã công bố trong khoa.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Báo cáo đề tài khoa'.
+2. Xem số lượng đề tài do GV ra đề và do SV đề xuất.</t>
+  </si>
+  <si>
+    <t>Báo cáo đề tài khoa</t>
+  </si>
+  <si>
+    <t>Thống kê rõ ràng tỷ lệ đề tài do GV đề xuất (80%) và SV tự đề xuất (20%), tỷ lệ duyệt thành công.</t>
+  </si>
+  <si>
+    <t>TC_GVK_014</t>
   </si>
   <si>
     <t>Danh sách SV</t>
@@ -2261,16 +2421,59 @@
   </si>
   <si>
     <t>1. Vào mục 'Danh sách Sinh viên'.
-2. Xem danh sách và thử tìm kiếm theo MSSV.</t>
+2. Xem danh sách hiển thị.</t>
   </si>
   <si>
     <t>GET /api/governance/students</t>
   </si>
   <si>
-    <t>Hiển thị danh sách SV: MSSV, Họ tên, Lớp niên chế, Email, Số điện thoại.</t>
-  </si>
-  <si>
-    <t>TC_GOV_007</t>
+    <t>Hiển thị danh sách SV khoa CNTT: MSSV, Họ tên, Lớp niên chế, Email, Số điện thoại.</t>
+  </si>
+  <si>
+    <t>TC_GVK_015</t>
+  </si>
+  <si>
+    <t>Tìm kiếm SV</t>
+  </si>
+  <si>
+    <t>Tìm kiếm sinh viên theo MSSV hoặc Họ tên</t>
+  </si>
+  <si>
+    <t>Tại danh sách sinh viên.</t>
+  </si>
+  <si>
+    <t>1. Nhập MSSV 'SV001'.
+2. Nhập tên 'Quang'.</t>
+  </si>
+  <si>
+    <t>Search: 'SV001'</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng sinh viên Trần Minh Quang khớp với từ khóa tìm kiếm.</t>
+  </si>
+  <si>
+    <t>TC_GVK_016</t>
+  </si>
+  <si>
+    <t>Lọc Khóa SV</t>
+  </si>
+  <si>
+    <t>Lọc danh sách sinh viên theo từng Khóa niên chế (K20, K21, K22)</t>
+  </si>
+  <si>
+    <t>Có sinh viên của nhiều khóa.</t>
+  </si>
+  <si>
+    <t>1. Chọn lọc theo Khóa 'K21'.</t>
+  </si>
+  <si>
+    <t>Filter: K21</t>
+  </si>
+  <si>
+    <t>Danh sách chỉ hiển thị các sinh viên thuộc khóa K21.</t>
+  </si>
+  <si>
+    <t>TC_GVK_017</t>
   </si>
   <si>
     <t>Danh sách GV</t>
@@ -2280,16 +2483,37 @@
   </si>
   <si>
     <t>1. Vào mục 'Danh sách Giảng viên'.
-2. Xem thông tin giảng viên.</t>
+2. Xem thông tin các giảng viên.</t>
   </si>
   <si>
     <t>GET /api/governance/lecturers</t>
   </si>
   <si>
-    <t>Hiển thị danh sách GV: Mã GV, Họ tên, Học vị, Chuyên môn, Số LHP đang phụ trách.</t>
-  </si>
-  <si>
-    <t>TC_GOV_008</t>
+    <t>Hiển thị: Mã GV, Họ tên, Học vị (ThS, TS, PGS), Chuyên môn nghiên cứu, Số lượng LHP đang phụ trách.</t>
+  </si>
+  <si>
+    <t>TC_GVK_018</t>
+  </si>
+  <si>
+    <t>Tìm kiếm GV</t>
+  </si>
+  <si>
+    <t>Tìm kiếm giảng viên theo Tên hoặc Chuyên môn</t>
+  </si>
+  <si>
+    <t>Tại danh sách giảng viên.</t>
+  </si>
+  <si>
+    <t>1. Nhập 'Trí tuệ nhân tạo' vào ô tìm kiếm chuyên môn.</t>
+  </si>
+  <si>
+    <t>Search: 'Trí tuệ nhân tạo'</t>
+  </si>
+  <si>
+    <t>Lọc ra các giảng viên có hướng nghiên cứu về Trí tuệ nhân tạo để dễ dàng phân công đồ án.</t>
+  </si>
+  <si>
+    <t>TC_GVK_019</t>
   </si>
   <si>
     <t>AI Phân tích</t>
@@ -2301,156 +2525,526 @@
     <t>Tại Dashboard Giáo vụ; có kết nối mạng.</t>
   </si>
   <si>
-    <t>1. Xem thẻ 'AI Phân tích khối lượng học vụ'.
+    <t>1. Xem thẻ 'AI Phân tích khối lượng học vụ khoa'.
 2. Bấm 'Phân tích ngay'.</t>
   </si>
   <si>
     <t>Gemini analyzeAcademicWorkload</t>
   </si>
   <si>
-    <t>AI phân tích tỷ lệ SV/GV, cảnh báo LHP bị quá tải và đề xuất cân đối số lượng nhóm đồ án.</t>
-  </si>
-  <si>
-    <t>TC_GOV_009</t>
-  </si>
-  <si>
-    <t>Xử lý khi AI Gemini phân tích bị gián đoạn mạng</t>
-  </si>
-  <si>
-    <t>Tắt mạng hoặc lỗi API Key.</t>
+    <t>AI phân tích tỷ lệ SV/GV, cảnh báo LHP bị quá tải sinh viên, khuyến nghị bổ sung GV hướng dẫn.</t>
+  </si>
+  <si>
+    <t>TC_GVK_020</t>
+  </si>
+  <si>
+    <t>Xử lý khi AI Gemini phân tích bị lỗi mạng hoặc timeout</t>
+  </si>
+  <si>
+    <t>Tắt mạng hoặc rút cáp USB.</t>
   </si>
   <si>
     <t>1. Bấm phân tích AI.</t>
   </si>
   <si>
-    <t>Offline</t>
-  </si>
-  <si>
-    <t>Thẻ AI hiển thị lỗi màu đỏ thân thiện: 'Không thể kết nối Gemini AI' kèm nút 'Thử lại'.</t>
-  </si>
-  <si>
-    <t>TC_GOV_010</t>
-  </si>
-  <si>
-    <t>Phòng Đào tạo</t>
-  </si>
-  <si>
-    <t>Giám sát số liệu đồ án toàn trường</t>
+    <t>Thẻ AI hiển thị lỗi màu đỏ thân thiện: 'Không thể kết nối Gemini AI' kèm nút 'Thử lại'. Không crash app.</t>
+  </si>
+  <si>
+    <t>TC_GVK_021</t>
+  </si>
+  <si>
+    <t>Cảnh báo trễ hạn</t>
+  </si>
+  <si>
+    <t>Giáo vụ xem danh sách các nhóm sinh viên chưa nộp báo cáo tiến độ</t>
+  </si>
+  <si>
+    <t>Có mốc báo cáo đã quá hạn nộp.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Theo dõi tiến độ đồ án khoa'.
+2. Lọc theo trạng thái 'Chưa nộp / Quá hạn'.</t>
+  </si>
+  <si>
+    <t>Filter: Overdue reports</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách các nhóm chưa nộp bài để giáo vụ gửi thông báo đôn đốc.</t>
+  </si>
+  <si>
+    <t>TC_GVK_022</t>
+  </si>
+  <si>
+    <t>Thông báo Khoa</t>
+  </si>
+  <si>
+    <t>Giáo vụ nhận thông báo khi có giảng viên mới được bổ sung</t>
+  </si>
+  <si>
+    <t>Admin vừa tạo tài khoản giảng viên mới cho khoa.</t>
+  </si>
+  <si>
+    <t>1. Vào mục Thông báo của Giáo vụ.
+2. Xem thông báo mới.</t>
+  </si>
+  <si>
+    <t>Nhận được thông báo: 'Tài khoản Giảng viên [Tên GV] vừa được kích hoạt thuộc khoa CNTT'.</t>
+  </si>
+  <si>
+    <t>TC_GVK_023</t>
+  </si>
+  <si>
+    <t>Hồ sơ Giáo vụ</t>
+  </si>
+  <si>
+    <t>Xem thông tin chi tiết và cập nhật Số điện thoại giáo vụ</t>
+  </si>
+  <si>
+    <t>Đăng nhập gvk.demo.</t>
+  </si>
+  <si>
+    <t>1. Vào trang Cá nhân.
+2. Chỉnh sửa số điện thoại liên hệ.
+3. Bấm Lưu.</t>
+  </si>
+  <si>
+    <t>Cập nhật thành công thông tin liên hệ giáo vụ khoa.</t>
+  </si>
+  <si>
+    <t>TC_GVK_024</t>
+  </si>
+  <si>
+    <t>Avatar Giáo vụ</t>
+  </si>
+  <si>
+    <t>Đổi ảnh đại diện cho tài khoản Giáo vụ khoa</t>
+  </si>
+  <si>
+    <t>Tại trang Cá nhân.</t>
+  </si>
+  <si>
+    <t>1. Bấm vào icon camera.
+2. Chọn ảnh chân dung từ thư viện máy.
+3. Tải lên.</t>
+  </si>
+  <si>
+    <t>Avatar upload</t>
+  </si>
+  <si>
+    <t>Ảnh tải lên thành công, cập nhật avatar giáo vụ trên toàn bộ giao diện.</t>
+  </si>
+  <si>
+    <t>TC_GVK_025</t>
+  </si>
+  <si>
+    <t>Bảo mật Khoa</t>
+  </si>
+  <si>
+    <t>Giáo vụ khoa chỉ được xem và phân công LHP thuộc khoa mình</t>
+  </si>
+  <si>
+    <t>Có LHP thuộc Khoa Ngoại ngữ hoặc Khoa Kinh tế.</t>
+  </si>
+  <si>
+    <t>1. Kiểm tra danh sách LHP hiển thị cho Giáo vụ CNTT.</t>
+  </si>
+  <si>
+    <t>Role scope check</t>
+  </si>
+  <si>
+    <t>Chỉ hiển thị các môn của khoa CNTT, không hiển thị và không sửa được LHP của khoa khác.</t>
+  </si>
+  <si>
+    <t>📋 KỊCH BẢN KIỂM THỬ PHÂN HỆ PHÒNG ĐÀO TẠO (ACADEMIC AFFAIRS)</t>
+  </si>
+  <si>
+    <t>TC_PDT_001</t>
+  </si>
+  <si>
+    <t>Dashboard Toàn trường</t>
+  </si>
+  <si>
+    <t>Giám sát số liệu đồ án tổng thể toàn trường (Liên khoa)</t>
   </si>
   <si>
     <t>Đăng nhập tài khoản pdt.demo.</t>
   </si>
   <si>
     <t>1. Vào Dashboard Phòng đào tạo.
-2. Quan sát số liệu đa khoa.</t>
-  </si>
-  <si>
-    <t>Hiển thị tổng thể toàn trường: tổng số LHP, tổng số sinh viên, tổng số đề tài được duyệt.</t>
-  </si>
-  <si>
-    <t>TC_GOV_011</t>
-  </si>
-  <si>
-    <t>AI Dự báo</t>
-  </si>
-  <si>
-    <t>Phòng đào tạo dùng AI dự báo xu hướng công nghệ đề tài</t>
+2. Quan sát số liệu tổng quan.</t>
+  </si>
+  <si>
+    <t>Hiển thị chuẩn xác: Tổng số Khoa, Tổng số LHP toàn trường, Tổng số SV làm đồ án, Tổng số đề tài được duyệt.</t>
+  </si>
+  <si>
+    <t>TC_PDT_002</t>
+  </si>
+  <si>
+    <t>Thống kê so sánh số lượng đồ án giữa các Khoa khác nhau</t>
+  </si>
+  <si>
+    <t>Hệ thống có dữ liệu của nhiều khoa.</t>
+  </si>
+  <si>
+    <t>1. Quan sát biểu đồ/thống kê phân bố theo khoa.</t>
+  </si>
+  <si>
+    <t>Department comparison</t>
+  </si>
+  <si>
+    <t>Hiển thị tỷ lệ số lượng đề tài giữa các khoa (CNTT: 60%, Điện tử: 25%, Kinh tế: 15%).</t>
+  </si>
+  <si>
+    <t>TC_PDT_003</t>
+  </si>
+  <si>
+    <t>Làm mới số liệu giám sát đào tạo cấp trường</t>
   </si>
   <si>
     <t>Tại Dashboard Phòng đào tạo.</t>
   </si>
   <si>
-    <t>1. Xem thẻ 'AI Dự báo đào tạo'.
-2. Đọc các khuyến nghị phân bổ.</t>
+    <t>1. Kéo vuốt màn hình từ trên xuống (Pull-to-refresh).</t>
+  </si>
+  <si>
+    <t>Tải lại toàn bộ số liệu thống kê liên khoa mới nhất từ CSDL.</t>
+  </si>
+  <si>
+    <t>TC_PDT_004</t>
+  </si>
+  <si>
+    <t>Cấu hình Học kỳ</t>
+  </si>
+  <si>
+    <t>Xem danh mục các Học kỳ và Năm học trong hệ thống</t>
+  </si>
+  <si>
+    <t>Đang ở quyền Phòng đào tạo.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Cấu hình học kỳ'.
+2. Xem danh sách học kỳ.</t>
+  </si>
+  <si>
+    <t>GET /api/semesters</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách học kỳ: HK1 2026-2027, HK2 2026-2027, HK Hè 2026-2027 kèm trạng thái Đang mở / Đã đóng.</t>
+  </si>
+  <si>
+    <t>TC_PDT_005</t>
+  </si>
+  <si>
+    <t>Thiết lập Học kỳ hiện tại (Active Semester) áp dụng toàn trường</t>
+  </si>
+  <si>
+    <t>Chuẩn bị bước sang học kỳ mới.</t>
+  </si>
+  <si>
+    <t>1. Chọn 'Học kỳ 1 2026-2027'.
+2. Thiết lập làm 'Học kỳ hiện tại'.
+3. Xác nhận.</t>
+  </si>
+  <si>
+    <t>Set Active Semester</t>
+  </si>
+  <si>
+    <t>Cập nhật thành công, tất cả các phân hệ khác (Sinh viên, Giảng viên, Giáo vụ) tự động đồng bộ theo học kỳ này.</t>
+  </si>
+  <si>
+    <t>TC_PDT_006</t>
+  </si>
+  <si>
+    <t>Khung thời gian</t>
+  </si>
+  <si>
+    <t>Xem khung thời gian kế hoạch đồ án toàn trường</t>
+  </si>
+  <si>
+    <t>Ở màn hình Kế hoạch đào tạo.</t>
+  </si>
+  <si>
+    <t>1. Xem các mốc: Bắt đầu đăng ký, Hạn nộp đề tài, Hạn nộp báo cáo, Tuần bảo vệ đồ án.</t>
+  </si>
+  <si>
+    <t>Training Schedule</t>
+  </si>
+  <si>
+    <t>Hiển thị lịch trình chuẩn mực theo quy chế đào tạo của nhà trường.</t>
+  </si>
+  <si>
+    <t>TC_PDT_007</t>
+  </si>
+  <si>
+    <t>Quản lý LHP cấp trường</t>
+  </si>
+  <si>
+    <t>Xem danh mục tất cả các LHP toàn trường (Liên khoa)</t>
+  </si>
+  <si>
+    <t>Tại mục 'Dữ liệu đào tạo'.</t>
+  </si>
+  <si>
+    <t>1. Vào xem danh sách LHP toàn trường.</t>
+  </si>
+  <si>
+    <t>GET /api/lop-hoc-phan (All departments)</t>
+  </si>
+  <si>
+    <t>Hiển thị toàn bộ LHP của các khoa với đầy đủ mã môn, giảng viên, sĩ số.</t>
+  </si>
+  <si>
+    <t>TC_PDT_008</t>
+  </si>
+  <si>
+    <t>Lọc LHP theo Khoa</t>
+  </si>
+  <si>
+    <t>Lọc danh sách LHP theo từng Khoa cụ thể</t>
+  </si>
+  <si>
+    <t>Tại danh sách LHP toàn trường.</t>
+  </si>
+  <si>
+    <t>1. Chọn lọc Khoa: 'Khoa Công nghệ thông tin'.
+2. Chọn lọc Khoa: 'Khoa Điện - Điện tử'.</t>
+  </si>
+  <si>
+    <t>Filter by Faculty</t>
+  </si>
+  <si>
+    <t>Danh sách lọc chuẩn xác các lớp thuộc về khoa đã chọn.</t>
+  </si>
+  <si>
+    <t>TC_PDT_009</t>
+  </si>
+  <si>
+    <t>Giám sát tiến độ</t>
+  </si>
+  <si>
+    <t>Giám sát các LHP chưa mở đợt đăng ký đồ án</t>
+  </si>
+  <si>
+    <t>Đã đến hạn mở đợt nhưng có lớp chưa mở.</t>
+  </si>
+  <si>
+    <t>1. Lọc LHP theo trạng thái 'Chưa mở đợt đăng ký'.</t>
+  </si>
+  <si>
+    <t>Filter: Pending batches</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách các lớp chưa mở đợt để phòng đào tạo nhắc nhở khoa đôn đốc giảng viên.</t>
+  </si>
+  <si>
+    <t>TC_PDT_010</t>
+  </si>
+  <si>
+    <t>Xem tỷ lệ sinh viên hoàn thành đồ án toàn trường</t>
+  </si>
+  <si>
+    <t>Nhiều lớp đã kết thúc chấm báo cáo.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Báo cáo tiến độ hoàn thành'.</t>
+  </si>
+  <si>
+    <t>Completion rate</t>
+  </si>
+  <si>
+    <t>Hiển thị tỷ lệ % sinh viên đạt yêu cầu đồ án so với tổng số sinh viên đăng ký.</t>
+  </si>
+  <si>
+    <t>TC_PDT_011</t>
+  </si>
+  <si>
+    <t>AI Dự báo đào tạo</t>
+  </si>
+  <si>
+    <t>Phòng đào tạo dùng AI Gemini dự báo nhu cầu đào tạo</t>
+  </si>
+  <si>
+    <t>Tại Dashboard Phòng đào tạo; có kết nối mạng.</t>
+  </si>
+  <si>
+    <t>1. Xem thẻ 'AI Dự báo đào tạo toàn trường'.
+2. Bấm 'Dự báo ngay'.</t>
   </si>
   <si>
     <t>Gemini analyzeTrainingForecast</t>
   </si>
   <si>
-    <t>AI phân tích xu hướng công nghệ (Mobile, AI, Cloud...) và đưa ra khuyến nghị phân bổ phòng lab/nhân lực.</t>
-  </si>
-  <si>
-    <t>TC_GOV_012</t>
-  </si>
-  <si>
-    <t>Cấu hình học kỳ</t>
-  </si>
-  <si>
-    <t>Xem danh mục các học kỳ và năm học trong hệ thống</t>
-  </si>
-  <si>
-    <t>Tại phân hệ Phòng đào tạo.</t>
-  </si>
-  <si>
-    <t>1. Vào mục 'Cấu hình học kỳ'.
-2. Xem danh sách các học kỳ.</t>
-  </si>
-  <si>
-    <t>GET /api/semesters</t>
-  </si>
-  <si>
-    <t>Hiển thị danh sách học kỳ (HK1 2026-2027, HK2 2026-2027) kèm thời gian hiệu lực.</t>
-  </si>
-  <si>
-    <t>TC_GOV_013</t>
-  </si>
-  <si>
-    <t>Chặn phân công trùng lặp cùng 1 giảng viên vào 1 LHP</t>
-  </si>
-  <si>
-    <t>GV A đã được phân công vào LHP X.</t>
-  </si>
-  <si>
-    <t>1. Thử chọn lại GV A để phân công vào LHP X lần nữa.</t>
-  </si>
-  <si>
-    <t>Duplicate assignment</t>
-  </si>
-  <si>
-    <t>Hệ thống thông báo: 'Giảng viên này đã được phân công cho lớp học phần từ trước'.</t>
-  </si>
-  <si>
-    <t>TC_GOV_014</t>
-  </si>
-  <si>
-    <t>Tra cứu SV</t>
-  </si>
-  <si>
-    <t>Lọc danh sách sinh viên theo từng Khóa niên chế (K20, K21, K22)</t>
-  </si>
-  <si>
-    <t>Ở màn hình danh sách SV.</t>
-  </si>
-  <si>
-    <t>1. Chọn lọc theo Khóa 'K21'.
-2. Quan sát danh sách.</t>
-  </si>
-  <si>
-    <t>Filter: K21</t>
-  </si>
-  <si>
-    <t>Danh sách chỉ hiển thị các sinh viên có MSSV bắt đầu bằng mã khóa K21.</t>
-  </si>
-  <si>
-    <t>TC_GOV_015</t>
-  </si>
-  <si>
-    <t>Thống kê đề tài</t>
-  </si>
-  <si>
-    <t>Giáo vụ xem báo cáo tổng hợp đề tài toàn khoa theo từng bộ môn</t>
-  </si>
-  <si>
-    <t>Tại Dashboard Giáo vụ.</t>
-  </si>
-  <si>
-    <t>1. Vào mục 'Báo cáo tổng hợp đề tài khoa'.</t>
-  </si>
-  <si>
-    <t>Báo cáo đề tài</t>
-  </si>
-  <si>
-    <t>Hiển thị chi tiết số lượng đề tài do GV đề xuất, số lượng đề tài do SV tự đề xuất, tỷ lệ đã duyệt.</t>
+    <t>AI phân tích xu hướng công nghệ (Flutter, AI, Cloud...) và đưa ra khuyến nghị phân bổ phòng lab/nhân lực.</t>
+  </si>
+  <si>
+    <t>TC_PDT_012</t>
+  </si>
+  <si>
+    <t>AI Dự báo công nghệ</t>
+  </si>
+  <si>
+    <t>AI phân tích xu hướng đề tài sinh viên quan tâm</t>
+  </si>
+  <si>
+    <t>Tại phần AI Dự báo.</t>
+  </si>
+  <si>
+    <t>1. Xem phân tích xu hướng đề tài từ AI.</t>
+  </si>
+  <si>
+    <t>AI technology trends</t>
+  </si>
+  <si>
+    <t>AI xếp hạng các công nghệ hot (AI: 40%, Mobile: 30%, Web: 20%) và gợi ý mở thêm lớp chuyên đề.</t>
+  </si>
+  <si>
+    <t>TC_PDT_013</t>
+  </si>
+  <si>
+    <t>AI Dự báo lỗi mạng</t>
+  </si>
+  <si>
+    <t>Xử lý khi AI Gemini dự báo gặp sự cố mất mạng</t>
+  </si>
+  <si>
+    <t>Ngắt kết nối mạng.</t>
+  </si>
+  <si>
+    <t>1. Bấm 'Dự báo ngay'.</t>
+  </si>
+  <si>
+    <t>Hiển thị thông báo lỗi màu đỏ kèm nút 'Thử lại'. Không bị văng ứng dụng.</t>
+  </si>
+  <si>
+    <t>TC_PDT_014</t>
+  </si>
+  <si>
+    <t>Toàn vẹn dữ liệu</t>
+  </si>
+  <si>
+    <t>Kiểm tra không có sinh viên mồ côi (không thuộc khoa nào)</t>
+  </si>
+  <si>
+    <t>Tại màn hình Dữ liệu đào tạo.</t>
+  </si>
+  <si>
+    <t>1. Kiểm tra thống kê sinh viên theo khoa.</t>
+  </si>
+  <si>
+    <t>Data integrity check</t>
+  </si>
+  <si>
+    <t>100% sinh viên đều được gán đúng vào một Khoa cụ thể trong CSDL.</t>
+  </si>
+  <si>
+    <t>TC_PDT_015</t>
+  </si>
+  <si>
+    <t>Quyền hạn độc lập</t>
+  </si>
+  <si>
+    <t>Phòng đào tạo chỉ có quyền giám sát, không can thiệp duyệt đề tài cụ thể của GV</t>
+  </si>
+  <si>
+    <t>Đăng nhập pdt.demo.</t>
+  </si>
+  <si>
+    <t>1. Thử tìm nút 'Duyệt đề tài' của một nhóm sinh viên cụ thể.</t>
+  </si>
+  <si>
+    <t>RBAC separation</t>
+  </si>
+  <si>
+    <t>Không có nút Duyệt/Từ chối đề tài (đảm bảo tính tự chủ học thuật của Giảng viên và Khoa).</t>
+  </si>
+  <si>
+    <t>TC_PDT_016</t>
+  </si>
+  <si>
+    <t>Báo cáo tổng kết</t>
+  </si>
+  <si>
+    <t>Xem bảng tổng hợp phổ điểm đồ án toàn trường</t>
+  </si>
+  <si>
+    <t>Đợt đồ án đã chấm xong.</t>
+  </si>
+  <si>
+    <t>1. Vào mục 'Phổ điểm đồ án toàn trường'.</t>
+  </si>
+  <si>
+    <t>Grade distribution</t>
+  </si>
+  <si>
+    <t>Hiển thị biểu đồ phân bổ điểm: Xuất sắc (9-10), Giỏi (8-8.9), Khá (7-7.9), Trung bình (5-6.9), Rớt (&lt;5).</t>
+  </si>
+  <si>
+    <t>TC_PDT_017</t>
+  </si>
+  <si>
+    <t>Thông báo Đào tạo</t>
+  </si>
+  <si>
+    <t>Nhận thông báo khi có đợt đăng ký đồ án mới được kích hoạt</t>
+  </si>
+  <si>
+    <t>Giảng viên vừa mở đợt đăng ký mới.</t>
+  </si>
+  <si>
+    <t>1. Vào mục Thông báo của Phòng đào tạo.</t>
+  </si>
+  <si>
+    <t>Hiện thông báo: 'Đợt đăng ký đồ án cho LHP [Tên LHP] vừa được kích hoạt'.</t>
+  </si>
+  <si>
+    <t>TC_PDT_018</t>
+  </si>
+  <si>
+    <t>Hồ sơ Đào tạo</t>
+  </si>
+  <si>
+    <t>Xem và cập nhật thông tin cán bộ Phòng đào tạo</t>
+  </si>
+  <si>
+    <t>1. Vào trang Cá nhân.
+2. Cập nhật Số điện thoại liên hệ.</t>
+  </si>
+  <si>
+    <t>Cập nhật thành công, thông tin lưu trữ an toàn vào Backend.</t>
+  </si>
+  <si>
+    <t>TC_PDT_019</t>
+  </si>
+  <si>
+    <t>Avatar Đào tạo</t>
+  </si>
+  <si>
+    <t>Đổi ảnh đại diện cho tài khoản Phòng đào tạo</t>
+  </si>
+  <si>
+    <t>1. Bấm icon camera &gt; Chọn ảnh.
+2. Xác nhận tải lên.</t>
+  </si>
+  <si>
+    <t>Ảnh đại diện cán bộ phòng đào tạo được cập nhật tức thì trên toàn bộ giao diện.</t>
+  </si>
+  <si>
+    <t>TC_PDT_020</t>
+  </si>
+  <si>
+    <t>Bảo mật Đào tạo</t>
+  </si>
+  <si>
+    <t>Chặn Phòng đào tạo truy cập các màn hình quản trị hệ thống của Admin</t>
+  </si>
+  <si>
+    <t>1. Thử tìm màn hình Quản lý User Admin hoặc gửi request POST /api/admin/users.</t>
+  </si>
+  <si>
+    <t>Access Admin API</t>
+  </si>
+  <si>
+    <t>Hệ thống từ chối với HTTP 403 Forbidden. Phân quyền vai trò tuyệt đối an toàn.</t>
   </si>
   <si>
     <t>📋 KỊCH BẢN KIỂM THỬ PHÂN HỆ QUẢN TRỊ VIÊN (ADMIN MODULE)</t>
@@ -3406,19 +4000,25 @@
     <t>4</t>
   </si>
   <si>
-    <t>5. Giáo vụ &amp; Đào tạo</t>
+    <t>5. Giáo vụ khoa</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>6. Quản trị hệ thống</t>
+    <t>6. Phòng đào tạo</t>
   </si>
   <si>
     <t>6</t>
   </si>
   <si>
-    <t>7. Phi chức năng &amp; Bảo mật</t>
+    <t>7. Quản trị hệ thống</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8. Phi chức năng &amp; Bảo mật</t>
   </si>
   <si>
     <t>TỔNG CỘNG TOÀN HỆ THỐNG</t>
@@ -3430,7 +4030,7 @@
     <t>Quy ước Trạng thái (Status):</t>
   </si>
   <si>
-    <t>• Pass: Tính năng chạy đúng 100% kết quả mong đợi. | • Fail: Có lỗi/sai logic/crash. | • Blocked: Bị nghẽn do lỗi module khác. | • Untested: Chưa kiểm tra.</t>
+    <t>• Pass: Tính năng chạy đúng 100% kết quả mong đợi. | • Fail: Có lỗi/sai logic/crash. | • Blocked: Bị nghéz do lỗi module khác. | • Untested: Chưa kiểm tra.</t>
   </si>
   <si>
     <t>Quy ước Mức độ nghiêm trọng (Severity):</t>
@@ -7790,7 +8390,7 @@
   <sheetPr>
     <tabColor rgb="FF059669"/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7910,28 +8510,28 @@
         <v>668</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>669</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>670</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>671</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="7" t="s">
         <v>672</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>673</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>674</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>35</v>
+      <c r="H4" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="6"/>
@@ -7941,31 +8541,31 @@
     </row>
     <row r="5" spans="1:14" ht="48" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>674</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>675</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>676</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>677</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>678</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>679</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>680</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>681</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>53</v>
+      <c r="H5" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="3"/>
@@ -7975,31 +8575,31 @@
     </row>
     <row r="6" spans="1:14" ht="48" customHeight="1">
       <c r="A6" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>682</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>683</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>684</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>685</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="F6" s="7" t="s">
         <v>686</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>687</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>688</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>22</v>
+      <c r="H6" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="6"/>
@@ -8009,28 +8609,28 @@
     </row>
     <row r="7" spans="1:14" ht="48" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>688</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>689</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>690</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>691</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>692</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>693</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>695</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>35</v>
+      <c r="H7" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>54</v>
@@ -8043,31 +8643,31 @@
     </row>
     <row r="8" spans="1:14" ht="48" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>696</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="F8" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>697</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>698</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>699</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>700</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>701</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>702</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>53</v>
+      <c r="H8" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="J8" s="7"/>
       <c r="K8" s="6"/>
@@ -8077,31 +8677,31 @@
     </row>
     <row r="9" spans="1:14" ht="48" customHeight="1">
       <c r="A9" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>699</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>700</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>701</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>702</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>703</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>704</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>705</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>699</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>706</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>707</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>708</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>53</v>
+      <c r="H9" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="J9" s="4"/>
       <c r="K9" s="3"/>
@@ -8111,25 +8711,25 @@
     </row>
     <row r="10" spans="1:14" ht="48" customHeight="1">
       <c r="A10" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>706</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>709</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>710</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>711</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>712</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>713</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>714</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>715</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>35</v>
@@ -8145,31 +8745,31 @@
     </row>
     <row r="11" spans="1:14" ht="48" customHeight="1">
       <c r="A11" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>712</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>713</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>714</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>715</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>716</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>710</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>717</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>718</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>719</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>720</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>721</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>53</v>
+      <c r="H11" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="3"/>
@@ -8179,31 +8779,31 @@
     </row>
     <row r="12" spans="1:14" ht="48" customHeight="1">
       <c r="A12" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>721</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>722</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="F12" s="7" t="s">
         <v>723</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>724</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>725</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>726</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>666</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>727</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>35</v>
+      <c r="H12" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="J12" s="7"/>
       <c r="K12" s="6"/>
@@ -8213,31 +8813,31 @@
     </row>
     <row r="13" spans="1:14" ht="48" customHeight="1">
       <c r="A13" s="3" t="s">
+        <v>725</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>726</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>727</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>728</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>729</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>730</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>731</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>732</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>733</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>53</v>
+      <c r="H13" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="3"/>
@@ -8247,31 +8847,31 @@
     </row>
     <row r="14" spans="1:14" ht="48" customHeight="1">
       <c r="A14" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>733</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>734</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>735</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="E14" s="7" t="s">
         <v>736</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="F14" s="7" t="s">
         <v>737</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>738</v>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>739</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>740</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>741</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>53</v>
+      <c r="H14" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="6"/>
@@ -8281,25 +8881,25 @@
     </row>
     <row r="15" spans="1:14" ht="48" customHeight="1">
       <c r="A15" s="3" t="s">
+        <v>739</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>740</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>741</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>742</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>683</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>743</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>744</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>745</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>746</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>747</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>35</v>
@@ -8315,25 +8915,25 @@
     </row>
     <row r="16" spans="1:14" ht="48" customHeight="1">
       <c r="A16" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>748</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="D16" s="7" t="s">
         <v>749</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>750</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>751</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>752</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>753</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>754</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>53</v>
@@ -8349,28 +8949,28 @@
     </row>
     <row r="17" spans="1:14" ht="48" customHeight="1">
       <c r="A17" s="3" t="s">
+        <v>753</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>754</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>755</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>756</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>757</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>758</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>759</v>
       </c>
-      <c r="F17" s="4" t="s">
-        <v>760</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>761</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>35</v>
+      <c r="H17" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>54</v>
@@ -8381,12 +8981,352 @@
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
+    <row r="18" spans="1:14" ht="48" customHeight="1">
+      <c r="A18" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>761</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>763</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>764</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>765</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J18" s="7"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+    </row>
+    <row r="19" spans="1:14" ht="48" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>768</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>769</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>749</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>771</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>772</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="1:14" ht="48" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>773</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>774</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>775</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>776</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>777</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>779</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J20" s="7"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+    </row>
+    <row r="21" spans="1:14" ht="48" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>781</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>784</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>785</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>786</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J21" s="4"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="1:14" ht="48" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>787</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>781</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>788</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>390</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>791</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J22" s="7"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+    </row>
+    <row r="23" spans="1:14" ht="48" customHeight="1">
+      <c r="A23" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>793</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>794</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>795</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>796</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>797</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>798</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J23" s="4"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+    </row>
+    <row r="24" spans="1:14" ht="48" customHeight="1">
+      <c r="A24" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>800</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>802</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>803</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="J24" s="7"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+    </row>
+    <row r="25" spans="1:14" ht="48" customHeight="1">
+      <c r="A25" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>806</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>807</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>808</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>809</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>810</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="1:14" ht="48" customHeight="1">
+      <c r="A26" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>812</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>813</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>814</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>815</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>816</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>817</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J26" s="7"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+    </row>
+    <row r="27" spans="1:14" ht="48" customHeight="1">
+      <c r="A27" s="3" t="s">
+        <v>818</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>819</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>820</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>821</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>823</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>824</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Trạng thái Test" prompt="Chọn: Pass, Fail, Blocked hoặc Untested" sqref="K3:K17">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Trạng thái Test" prompt="Chọn: Pass, Fail, Blocked hoặc Untested" sqref="K3:K27">
       <formula1>"Pass,Fail,Blocked,Untested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8395,6 +9335,785 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FFD97706"/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="25.7109375" customWidth="1"/>
+    <col min="5" max="5" width="34.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" customWidth="1"/>
+    <col min="7" max="7" width="34.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="26.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="13" max="13" width="14.7109375" customWidth="1"/>
+    <col min="14" max="14" width="13.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="32" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>825</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" ht="28" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="48" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>826</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>827</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>828</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>829</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>830</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>831</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="4"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+    </row>
+    <row r="4" spans="1:14" ht="48" customHeight="1">
+      <c r="A4" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>827</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>833</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>834</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>835</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>836</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>837</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="7"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+    </row>
+    <row r="5" spans="1:14" ht="48" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>838</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>827</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>839</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>840</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>841</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>842</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J5" s="4"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" ht="48" customHeight="1">
+      <c r="A6" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>844</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>845</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>846</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>847</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>848</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>849</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+    </row>
+    <row r="7" spans="1:14" ht="48" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>850</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>844</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>851</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>852</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>853</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>854</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>855</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+    </row>
+    <row r="8" spans="1:14" ht="48" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>856</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>857</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>858</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>859</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>860</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>861</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>862</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="7"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+    </row>
+    <row r="9" spans="1:14" ht="48" customHeight="1">
+      <c r="A9" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>866</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>867</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>868</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>869</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="4"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" ht="48" customHeight="1">
+      <c r="A10" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>872</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>873</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>874</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>875</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>876</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" s="7"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+    </row>
+    <row r="11" spans="1:14" ht="48" customHeight="1">
+      <c r="A11" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>878</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>879</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>880</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>881</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>882</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>883</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+    </row>
+    <row r="12" spans="1:14" ht="48" customHeight="1">
+      <c r="A12" s="6" t="s">
+        <v>884</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>878</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>886</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>887</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>888</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>889</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J12" s="7"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+    </row>
+    <row r="13" spans="1:14" ht="48" customHeight="1">
+      <c r="A13" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>891</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>892</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>893</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>894</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>896</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J13" s="4"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:14" ht="48" customHeight="1">
+      <c r="A14" s="6" t="s">
+        <v>897</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>898</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>899</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>900</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>901</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>902</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>903</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="J14" s="7"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+    </row>
+    <row r="15" spans="1:14" ht="48" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>905</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>906</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>907</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>908</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J15" s="4"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" ht="48" customHeight="1">
+      <c r="A16" s="6" t="s">
+        <v>910</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>911</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>912</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>913</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>914</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>915</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>916</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" s="7"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+    </row>
+    <row r="17" spans="1:14" ht="48" customHeight="1">
+      <c r="A17" s="3" t="s">
+        <v>917</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>918</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>919</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>920</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>921</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>922</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>923</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="1:14" ht="48" customHeight="1">
+      <c r="A18" s="6" t="s">
+        <v>924</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>925</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>926</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>927</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>928</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>929</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>930</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J18" s="7"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+    </row>
+    <row r="19" spans="1:14" ht="48" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>932</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>933</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>934</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>935</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>936</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="1:14" ht="48" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>937</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>938</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>920</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>941</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="7"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+    </row>
+    <row r="21" spans="1:14" ht="48" customHeight="1">
+      <c r="A21" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>943</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>944</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>814</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>945</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>816</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>946</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J21" s="4"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="1:14" ht="48" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>947</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>948</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>920</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>951</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>952</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Trạng thái Test" prompt="Chọn: Pass, Fail, Blocked hoặc Untested" sqref="K3:K22">
+      <formula1>"Pass,Fail,Blocked,Untested"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF7C3AED"/>
@@ -8420,7 +10139,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>762</v>
+        <v>953</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -8482,25 +10201,25 @@
     </row>
     <row r="3" spans="1:14" ht="48" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>763</v>
+        <v>954</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>764</v>
+        <v>955</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>765</v>
+        <v>956</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>766</v>
+        <v>957</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>767</v>
+        <v>958</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>666</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>768</v>
+        <v>959</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>35</v>
@@ -8516,25 +10235,25 @@
     </row>
     <row r="4" spans="1:14" ht="48" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>769</v>
+        <v>960</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>770</v>
+        <v>961</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>771</v>
+        <v>962</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>772</v>
+        <v>963</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>773</v>
+        <v>964</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>774</v>
+        <v>965</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>775</v>
+        <v>966</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>35</v>
@@ -8550,25 +10269,25 @@
     </row>
     <row r="5" spans="1:14" ht="48" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>776</v>
+        <v>967</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>777</v>
+        <v>968</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>778</v>
+        <v>969</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>779</v>
+        <v>970</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>780</v>
+        <v>971</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>781</v>
+        <v>972</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>782</v>
+        <v>973</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>35</v>
@@ -8584,25 +10303,25 @@
     </row>
     <row r="6" spans="1:14" ht="48" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>783</v>
+        <v>974</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>784</v>
+        <v>975</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>785</v>
+        <v>976</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>786</v>
+        <v>977</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>787</v>
+        <v>978</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>788</v>
+        <v>979</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>789</v>
+        <v>980</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>35</v>
@@ -8618,25 +10337,25 @@
     </row>
     <row r="7" spans="1:14" ht="48" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>790</v>
+        <v>981</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>791</v>
+        <v>982</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>792</v>
+        <v>983</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>793</v>
+        <v>984</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>794</v>
+        <v>985</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>795</v>
+        <v>986</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>796</v>
+        <v>987</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>35</v>
@@ -8652,25 +10371,25 @@
     </row>
     <row r="8" spans="1:14" ht="48" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>797</v>
+        <v>988</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>798</v>
+        <v>989</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>799</v>
+        <v>990</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>800</v>
+        <v>991</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>801</v>
+        <v>992</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>802</v>
+        <v>993</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>803</v>
+        <v>994</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>22</v>
@@ -8686,25 +10405,25 @@
     </row>
     <row r="9" spans="1:14" ht="48" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>804</v>
+        <v>995</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>805</v>
+        <v>996</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>806</v>
+        <v>997</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>807</v>
+        <v>998</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>808</v>
+        <v>999</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>809</v>
+        <v>1000</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>810</v>
+        <v>1001</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>35</v>
@@ -8720,25 +10439,25 @@
     </row>
     <row r="10" spans="1:14" ht="48" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>811</v>
+        <v>1002</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>805</v>
+        <v>996</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>812</v>
+        <v>1003</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>813</v>
+        <v>1004</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>814</v>
+        <v>1005</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>815</v>
+        <v>1006</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>816</v>
+        <v>1007</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>53</v>
@@ -8754,25 +10473,25 @@
     </row>
     <row r="11" spans="1:14" ht="48" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>817</v>
+        <v>1008</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>818</v>
+        <v>1009</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>819</v>
+        <v>1010</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>820</v>
+        <v>1011</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>821</v>
+        <v>1012</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>822</v>
+        <v>1013</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>823</v>
+        <v>1014</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>35</v>
@@ -8788,25 +10507,25 @@
     </row>
     <row r="12" spans="1:14" ht="48" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>824</v>
+        <v>1015</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>825</v>
+        <v>1016</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>826</v>
+        <v>1017</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>827</v>
+        <v>1018</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>828</v>
+        <v>1019</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>829</v>
+        <v>1020</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>830</v>
+        <v>1021</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>35</v>
@@ -8822,25 +10541,25 @@
     </row>
     <row r="13" spans="1:14" ht="48" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>831</v>
+        <v>1022</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>832</v>
+        <v>1023</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>833</v>
+        <v>1024</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>834</v>
+        <v>1025</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>835</v>
+        <v>1026</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>836</v>
+        <v>1027</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>837</v>
+        <v>1028</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>35</v>
@@ -8856,25 +10575,25 @@
     </row>
     <row r="14" spans="1:14" ht="48" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>838</v>
+        <v>1029</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>840</v>
+        <v>1031</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>841</v>
+        <v>1032</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>842</v>
+        <v>1033</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>843</v>
+        <v>1034</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>844</v>
+        <v>1035</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>35</v>
@@ -8890,25 +10609,25 @@
     </row>
     <row r="15" spans="1:14" ht="48" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>845</v>
+        <v>1036</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>846</v>
+        <v>1037</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>847</v>
+        <v>1038</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>848</v>
+        <v>1039</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>849</v>
+        <v>1040</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>850</v>
+        <v>1041</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>35</v>
@@ -8924,25 +10643,25 @@
     </row>
     <row r="16" spans="1:14" ht="48" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>851</v>
+        <v>1042</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>852</v>
+        <v>1043</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>853</v>
+        <v>1044</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>854</v>
+        <v>1045</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>855</v>
+        <v>1046</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>856</v>
+        <v>1047</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>35</v>
@@ -8958,25 +10677,25 @@
     </row>
     <row r="17" spans="1:14" ht="48" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>857</v>
+        <v>1048</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>858</v>
+        <v>1049</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>859</v>
+        <v>1050</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>860</v>
+        <v>1051</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>861</v>
+        <v>1052</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>862</v>
+        <v>1053</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>22</v>
@@ -8992,25 +10711,25 @@
     </row>
     <row r="18" spans="1:14" ht="48" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>863</v>
+        <v>1054</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>864</v>
+        <v>1055</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>865</v>
+        <v>1056</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>866</v>
+        <v>1057</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>867</v>
+        <v>1058</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>868</v>
+        <v>1059</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>35</v>
@@ -9026,25 +10745,25 @@
     </row>
     <row r="19" spans="1:14" ht="48" customHeight="1">
       <c r="A19" s="3" t="s">
-        <v>869</v>
+        <v>1060</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>870</v>
+        <v>1061</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>871</v>
+        <v>1062</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>872</v>
+        <v>1063</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>873</v>
+        <v>1064</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>874</v>
+        <v>1065</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>53</v>
@@ -9060,25 +10779,25 @@
     </row>
     <row r="20" spans="1:14" ht="48" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>875</v>
+        <v>1066</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>876</v>
+        <v>1067</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>877</v>
+        <v>1068</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>878</v>
+        <v>1069</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>879</v>
+        <v>1070</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>880</v>
+        <v>1071</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>881</v>
+        <v>1072</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>53</v>
@@ -9094,25 +10813,25 @@
     </row>
     <row r="21" spans="1:14" ht="48" customHeight="1">
       <c r="A21" s="3" t="s">
-        <v>882</v>
+        <v>1073</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>883</v>
+        <v>1074</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>884</v>
+        <v>1075</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>813</v>
+        <v>1004</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>885</v>
+        <v>1076</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>886</v>
+        <v>1077</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>887</v>
+        <v>1078</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>53</v>
@@ -9128,25 +10847,25 @@
     </row>
     <row r="22" spans="1:14" ht="48" customHeight="1">
       <c r="A22" s="6" t="s">
-        <v>888</v>
+        <v>1079</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>889</v>
+        <v>1080</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>890</v>
+        <v>1081</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>891</v>
+        <v>1082</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>892</v>
+        <v>1083</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>893</v>
+        <v>1084</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>53</v>
@@ -9162,25 +10881,25 @@
     </row>
     <row r="23" spans="1:14" ht="48" customHeight="1">
       <c r="A23" s="3" t="s">
-        <v>894</v>
+        <v>1085</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>839</v>
+        <v>1030</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>895</v>
+        <v>1086</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>896</v>
+        <v>1087</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>897</v>
+        <v>1088</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>898</v>
+        <v>1089</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>899</v>
+        <v>1090</v>
       </c>
       <c r="H23" s="8" t="s">
         <v>35</v>
@@ -9196,25 +10915,25 @@
     </row>
     <row r="24" spans="1:14" ht="48" customHeight="1">
       <c r="A24" s="6" t="s">
-        <v>900</v>
+        <v>1091</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>901</v>
+        <v>1092</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>902</v>
+        <v>1093</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>903</v>
+        <v>1094</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>904</v>
+        <v>1095</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>905</v>
+        <v>1096</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>906</v>
+        <v>1097</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>35</v>
@@ -9230,25 +10949,25 @@
     </row>
     <row r="25" spans="1:14" ht="48" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>907</v>
+        <v>1098</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>908</v>
+        <v>1099</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>909</v>
+        <v>1100</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>910</v>
+        <v>1101</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>911</v>
+        <v>1102</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>912</v>
+        <v>1103</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>913</v>
+        <v>1104</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>22</v>
@@ -9264,25 +10983,25 @@
     </row>
     <row r="26" spans="1:14" ht="48" customHeight="1">
       <c r="A26" s="6" t="s">
-        <v>914</v>
+        <v>1105</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>915</v>
+        <v>1106</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>916</v>
+        <v>1107</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>917</v>
+        <v>1108</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>918</v>
+        <v>1109</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>919</v>
+        <v>1110</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>920</v>
+        <v>1111</v>
       </c>
       <c r="H26" s="9" t="s">
         <v>53</v>
@@ -9309,7 +11028,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF334155"/>
@@ -9335,7 +11054,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="32" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>921</v>
+        <v>1112</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -9397,25 +11116,25 @@
     </row>
     <row r="3" spans="1:14" ht="48" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>922</v>
+        <v>1113</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>923</v>
+        <v>1114</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>924</v>
+        <v>1115</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>925</v>
+        <v>1116</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>926</v>
+        <v>1117</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>927</v>
+        <v>1118</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>928</v>
+        <v>1119</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>22</v>
@@ -9431,25 +11150,25 @@
     </row>
     <row r="4" spans="1:14" ht="48" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>929</v>
+        <v>1120</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>930</v>
+        <v>1121</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>931</v>
+        <v>1122</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>932</v>
+        <v>1123</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>933</v>
+        <v>1124</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>934</v>
+        <v>1125</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>935</v>
+        <v>1126</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>22</v>
@@ -9465,25 +11184,25 @@
     </row>
     <row r="5" spans="1:14" ht="48" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>936</v>
+        <v>1127</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>937</v>
+        <v>1128</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>938</v>
+        <v>1129</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>939</v>
+        <v>1130</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>940</v>
+        <v>1131</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>941</v>
+        <v>1132</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>942</v>
+        <v>1133</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>22</v>
@@ -9499,25 +11218,25 @@
     </row>
     <row r="6" spans="1:14" ht="48" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>943</v>
+        <v>1134</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>937</v>
+        <v>1128</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>944</v>
+        <v>1135</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>945</v>
+        <v>1136</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>946</v>
+        <v>1137</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>947</v>
+        <v>1138</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>948</v>
+        <v>1139</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>22</v>
@@ -9533,25 +11252,25 @@
     </row>
     <row r="7" spans="1:14" ht="48" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>949</v>
+        <v>1140</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>950</v>
+        <v>1141</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>951</v>
+        <v>1142</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>952</v>
+        <v>1143</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>953</v>
+        <v>1144</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>954</v>
+        <v>1145</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>955</v>
+        <v>1146</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>35</v>
@@ -9567,25 +11286,25 @@
     </row>
     <row r="8" spans="1:14" ht="48" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>956</v>
+        <v>1147</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>957</v>
+        <v>1148</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>958</v>
+        <v>1149</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>959</v>
+        <v>1150</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>960</v>
+        <v>1151</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>961</v>
+        <v>1152</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>962</v>
+        <v>1153</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>53</v>
@@ -9601,25 +11320,25 @@
     </row>
     <row r="9" spans="1:14" ht="48" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>963</v>
+        <v>1154</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>964</v>
+        <v>1155</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>965</v>
+        <v>1156</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>966</v>
+        <v>1157</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>967</v>
+        <v>1158</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>968</v>
+        <v>1159</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>969</v>
+        <v>1160</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>53</v>
@@ -9635,25 +11354,25 @@
     </row>
     <row r="10" spans="1:14" ht="48" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>970</v>
+        <v>1161</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>971</v>
+        <v>1162</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>972</v>
+        <v>1163</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>973</v>
+        <v>1164</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>974</v>
+        <v>1165</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>975</v>
+        <v>1166</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>976</v>
+        <v>1167</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>35</v>
@@ -9669,25 +11388,25 @@
     </row>
     <row r="11" spans="1:14" ht="48" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>977</v>
+        <v>1168</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>978</v>
+        <v>1169</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>979</v>
+        <v>1170</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>980</v>
+        <v>1171</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>981</v>
+        <v>1172</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>982</v>
+        <v>1173</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>983</v>
+        <v>1174</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>97</v>
@@ -9703,25 +11422,25 @@
     </row>
     <row r="12" spans="1:14" ht="48" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>984</v>
+        <v>1175</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>985</v>
+        <v>1176</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>986</v>
+        <v>1177</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>987</v>
+        <v>1178</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>988</v>
+        <v>1179</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>989</v>
+        <v>1180</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>990</v>
+        <v>1181</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>35</v>
@@ -9737,25 +11456,25 @@
     </row>
     <row r="13" spans="1:14" ht="48" customHeight="1">
       <c r="A13" s="3" t="s">
-        <v>991</v>
+        <v>1182</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>992</v>
+        <v>1183</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>993</v>
+        <v>1184</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>994</v>
+        <v>1185</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>995</v>
+        <v>1186</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>996</v>
+        <v>1187</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>997</v>
+        <v>1188</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>35</v>
@@ -9771,25 +11490,25 @@
     </row>
     <row r="14" spans="1:14" ht="48" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>998</v>
+        <v>1189</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>999</v>
+        <v>1190</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>1000</v>
+        <v>1191</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>1001</v>
+        <v>1192</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>1002</v>
+        <v>1193</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>1003</v>
+        <v>1194</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>1004</v>
+        <v>1195</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>22</v>
@@ -9805,25 +11524,25 @@
     </row>
     <row r="15" spans="1:14" ht="48" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>1005</v>
+        <v>1196</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>1006</v>
+        <v>1197</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>1007</v>
+        <v>1198</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>1008</v>
+        <v>1199</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>1009</v>
+        <v>1200</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>1010</v>
+        <v>1201</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>1011</v>
+        <v>1202</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>53</v>
@@ -9839,25 +11558,25 @@
     </row>
     <row r="16" spans="1:14" ht="48" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>1012</v>
+        <v>1203</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>1013</v>
+        <v>1204</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>1014</v>
+        <v>1205</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>1015</v>
+        <v>1206</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>1016</v>
+        <v>1207</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>1017</v>
+        <v>1208</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>1018</v>
+        <v>1209</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>53</v>
@@ -9873,25 +11592,25 @@
     </row>
     <row r="17" spans="1:14" ht="48" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>1019</v>
+        <v>1210</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>1020</v>
+        <v>1211</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>1021</v>
+        <v>1212</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>1022</v>
+        <v>1213</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>1023</v>
+        <v>1214</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>1024</v>
+        <v>1215</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>1025</v>
+        <v>1216</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>53</v>
@@ -9907,25 +11626,25 @@
     </row>
     <row r="18" spans="1:14" ht="48" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>1026</v>
+        <v>1217</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>1027</v>
+        <v>1218</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>1028</v>
+        <v>1219</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>1029</v>
+        <v>1220</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>1030</v>
+        <v>1221</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>1031</v>
+        <v>1222</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>1032</v>
+        <v>1223</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>35</v>
@@ -9952,12 +11671,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF1E3A5F"/>
   </sheetPr>
-  <dimension ref="B2:I30"/>
+  <dimension ref="B2:I31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -9969,7 +11688,7 @@
   <sheetData>
     <row r="2" spans="2:8" ht="35" customHeight="1">
       <c r="B2" s="1" t="s">
-        <v>1033</v>
+        <v>1224</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -9980,7 +11699,7 @@
     </row>
     <row r="3" spans="2:8" ht="20" customHeight="1">
       <c r="B3" s="11" t="s">
-        <v>1034</v>
+        <v>1225</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -9991,77 +11710,77 @@
     </row>
     <row r="5" spans="2:8">
       <c r="B5" s="12" t="s">
-        <v>1035</v>
+        <v>1226</v>
       </c>
       <c r="C5" s="12"/>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="13" t="s">
-        <v>1036</v>
+        <v>1227</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1037</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="7" spans="2:8">
       <c r="B7" s="13" t="s">
-        <v>1038</v>
+        <v>1229</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1039</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="8" spans="2:8">
       <c r="B8" s="13" t="s">
-        <v>1040</v>
+        <v>1231</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1041</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="13" t="s">
-        <v>1042</v>
+        <v>1233</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1043</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="13" t="s">
-        <v>1044</v>
+        <v>1235</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1045</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="13" t="s">
-        <v>1046</v>
+        <v>1237</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1047</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="12" spans="2:8">
       <c r="B12" s="13" t="s">
-        <v>1048</v>
+        <v>1239</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1049</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="13" t="s">
-        <v>1050</v>
+        <v>1241</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>1051</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="15" spans="2:8">
       <c r="B15" s="12" t="s">
-        <v>1052</v>
+        <v>1243</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -10072,36 +11791,36 @@
     </row>
     <row r="17" spans="2:9">
       <c r="B17" s="2" t="s">
-        <v>1053</v>
+        <v>1244</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>1054</v>
+        <v>1245</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>1055</v>
+        <v>1246</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>1056</v>
+        <v>1247</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>1057</v>
+        <v>1248</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>1058</v>
+        <v>1249</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>1059</v>
+        <v>1250</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>1060</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="3" t="s">
-        <v>1061</v>
+        <v>1252</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>1062</v>
+        <v>1253</v>
       </c>
       <c r="D18" s="15">
         <v>28</v>
@@ -10129,10 +11848,10 @@
     </row>
     <row r="19" spans="2:9">
       <c r="B19" s="3" t="s">
-        <v>1063</v>
+        <v>1254</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>1064</v>
+        <v>1255</v>
       </c>
       <c r="D19" s="15">
         <v>44</v>
@@ -10160,10 +11879,10 @@
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="3" t="s">
-        <v>1065</v>
+        <v>1256</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>1066</v>
+        <v>1257</v>
       </c>
       <c r="D20" s="15">
         <v>30</v>
@@ -10191,24 +11910,24 @@
     </row>
     <row r="21" spans="2:9">
       <c r="B21" s="3" t="s">
-        <v>1067</v>
+        <v>1258</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>1068</v>
+        <v>1259</v>
       </c>
       <c r="D21" s="15">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E21" s="3">
-        <f>COUNTIF('5. Giáo vụ &amp; Đào tạo'!K3:K17, "Pass")</f>
+        <f>COUNTIF('5. Giáo vụ khoa'!K3:K27, "Pass")</f>
         <v>0</v>
       </c>
       <c r="F21" s="3">
-        <f>COUNTIF('5. Giáo vụ &amp; Đào tạo'!K3:K17, "Fail")</f>
+        <f>COUNTIF('5. Giáo vụ khoa'!K3:K27, "Fail")</f>
         <v>0</v>
       </c>
       <c r="G21" s="3">
-        <f>COUNTIF('5. Giáo vụ &amp; Đào tạo'!K3:K17, "Blocked")</f>
+        <f>COUNTIF('5. Giáo vụ khoa'!K3:K27, "Blocked")</f>
         <v>0</v>
       </c>
       <c r="H21" s="3">
@@ -10222,24 +11941,24 @@
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="3" t="s">
-        <v>1069</v>
+        <v>1260</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>1070</v>
+        <v>1261</v>
       </c>
       <c r="D22" s="15">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E22" s="3">
-        <f>COUNTIF('6. Quản trị hệ thống'!K3:K26, "Pass")</f>
+        <f>COUNTIF('6. Phòng đào tạo'!K3:K22, "Pass")</f>
         <v>0</v>
       </c>
       <c r="F22" s="3">
-        <f>COUNTIF('6. Quản trị hệ thống'!K3:K26, "Fail")</f>
+        <f>COUNTIF('6. Phòng đào tạo'!K3:K22, "Fail")</f>
         <v>0</v>
       </c>
       <c r="G22" s="3">
-        <f>COUNTIF('6. Quản trị hệ thống'!K3:K26, "Blocked")</f>
+        <f>COUNTIF('6. Phòng đào tạo'!K3:K22, "Blocked")</f>
         <v>0</v>
       </c>
       <c r="H22" s="3">
@@ -10253,24 +11972,24 @@
     </row>
     <row r="23" spans="2:9">
       <c r="B23" s="3" t="s">
-        <v>1071</v>
+        <v>1262</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>1072</v>
+        <v>1263</v>
       </c>
       <c r="D23" s="15">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E23" s="3">
-        <f>COUNTIF('7. Phi chức năng &amp; Bảo mật'!K3:K18, "Pass")</f>
+        <f>COUNTIF('7. Quản trị hệ thống'!K3:K26, "Pass")</f>
         <v>0</v>
       </c>
       <c r="F23" s="3">
-        <f>COUNTIF('7. Phi chức năng &amp; Bảo mật'!K3:K18, "Fail")</f>
+        <f>COUNTIF('7. Quản trị hệ thống'!K3:K26, "Fail")</f>
         <v>0</v>
       </c>
       <c r="G23" s="3">
-        <f>COUNTIF('7. Phi chức năng &amp; Bảo mật'!K3:K18, "Blocked")</f>
+        <f>COUNTIF('7. Quản trị hệ thống'!K3:K26, "Blocked")</f>
         <v>0</v>
       </c>
       <c r="H23" s="3">
@@ -10283,67 +12002,84 @@
       </c>
     </row>
     <row r="24" spans="2:9">
-      <c r="B24" s="2" t="s">
-        <v>1073</v>
-      </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2">
-        <f>SUM(D18:D23)</f>
+      <c r="B24" s="3" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>1265</v>
+      </c>
+      <c r="D24" s="15">
+        <v>16</v>
+      </c>
+      <c r="E24" s="3">
+        <f>COUNTIF('8. Phi chức năng &amp; Bảo mật'!K3:K18, "Pass")</f>
         <v>0</v>
       </c>
-      <c r="E24" s="2">
-        <f>SUM(E18:E23)</f>
+      <c r="F24" s="3">
+        <f>COUNTIF('8. Phi chức năng &amp; Bảo mật'!K3:K18, "Fail")</f>
         <v>0</v>
       </c>
-      <c r="F24" s="2">
-        <f>SUM(F18:F23)</f>
+      <c r="G24" s="3">
+        <f>COUNTIF('8. Phi chức năng &amp; Bảo mật'!K3:K18, "Blocked")</f>
         <v>0</v>
       </c>
-      <c r="G24" s="2">
-        <f>SUM(G18:G23)</f>
+      <c r="H24" s="3">
+        <f>D24-E24-F24-G24</f>
         <v>0</v>
       </c>
-      <c r="H24" s="2">
-        <f>SUM(H18:H23)</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="17">
+      <c r="I24" s="16">
         <f>IF(D24&gt;0, E24/D24, 0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:9">
-      <c r="B26" s="12" t="s">
-        <v>1074</v>
-      </c>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
+    <row r="25" spans="2:9">
+      <c r="B25" s="2" t="s">
+        <v>1266</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2">
+        <f>SUM(D18:D24)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="2">
+        <f>SUM(E18:E24)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="2">
+        <f>SUM(F18:F24)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="2">
+        <f>SUM(G18:G24)</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="2">
+        <f>SUM(H18:H24)</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="17">
+        <f>IF(D25&gt;0, E25/D25, 0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="2:9">
-      <c r="B27" s="13" t="s">
-        <v>1075</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>1076</v>
-      </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
+      <c r="B27" s="12" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
     </row>
     <row r="28" spans="2:9">
       <c r="B28" s="13" t="s">
-        <v>1077</v>
+        <v>1268</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>1078</v>
+        <v>1269</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
@@ -10354,10 +12090,10 @@
     </row>
     <row r="29" spans="2:9">
       <c r="B29" s="13" t="s">
-        <v>1079</v>
+        <v>1270</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>1080</v>
+        <v>1271</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
@@ -10368,10 +12104,10 @@
     </row>
     <row r="30" spans="2:9">
       <c r="B30" s="13" t="s">
-        <v>1081</v>
+        <v>1272</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>1082</v>
+        <v>1273</v>
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="14"/>
@@ -10380,18 +12116,32 @@
       <c r="H30" s="14"/>
       <c r="I30" s="14"/>
     </row>
+    <row r="31" spans="2:9">
+      <c r="B31" s="13" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="C27:I27"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:I27"/>
     <mergeCell ref="C28:I28"/>
     <mergeCell ref="C29:I29"/>
     <mergeCell ref="C30:I30"/>
+    <mergeCell ref="C31:I31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>